<commit_message>
update Sat 05/30/2026 04:06:00
</commit_message>
<xml_diff>
--- a/Green/class_attendance_data.xlsx
+++ b/Green/class_attendance_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -740,6 +740,286 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>მოსწავლე 11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>91</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>გაუმჯობესება</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>M-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>მოსწავლე 12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>71%</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" t="n">
+        <v>50</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>კლება</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>M-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>მოსწავლე 13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>89%</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E14" t="n">
+        <v>83</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>სტაბილური</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>M-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>მოსწავლე 14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>42</v>
+      </c>
+      <c r="E15" t="n">
+        <v>45</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>კლება</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>M-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>მოსწავლე 15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>96%</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>გაუმჯობესება</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>M-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>მოსწავლე 16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>28</v>
+      </c>
+      <c r="E17" t="n">
+        <v>60</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>კლება</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>M-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>მოსწავლე 17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" t="n">
+        <v>84</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>სტაბილური</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>M-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>მოსწავლე 18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>84%</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>19</v>
+      </c>
+      <c r="E19" t="n">
+        <v>75</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>გაუმჯობესება</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>M-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>მოსწავლე 19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>97%</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>96</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>სტაბილური</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>M-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>მოსწავლე 20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>79%</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>24</v>
+      </c>
+      <c r="E21" t="n">
+        <v>67</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>გაუმჯობესება</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>